<commit_message>
feat: re-arrange teachers according to staff details excel column 1 (start) and map photos to column 2 (serial)
</commit_message>
<xml_diff>
--- a/staff/staff details.xlsx
+++ b/staff/staff details.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$38</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="91">
   <si>
     <t>Name</t>
   </si>
@@ -292,6 +292,9 @@
   </si>
   <si>
     <t>B.SC/M.SC</t>
+  </si>
+  <si>
+    <t>start</t>
   </si>
 </sst>
 </file>
@@ -550,33 +553,14 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
   <dxfs count="11">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -741,6 +725,15 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -748,18 +741,28 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -776,16 +779,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:G38" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="9" tableBorderDxfId="10" totalsRowBorderDxfId="8" headerRowCellStyle="Output">
-  <autoFilter ref="A1:G38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="B1:H38" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8" totalsRowBorderDxfId="7" headerRowCellStyle="Output">
+  <autoFilter ref="B1:H38"/>
+  <sortState ref="B2:H38">
+    <sortCondition ref="B1:B38"/>
+  </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" name="SERIAL" dataDxfId="7" dataCellStyle="Output"/>
-    <tableColumn id="2" name="Name" dataDxfId="6" dataCellStyle="Output"/>
-    <tableColumn id="3" name="Post" dataDxfId="5"/>
-    <tableColumn id="4" name="Subject" dataDxfId="4" dataCellStyle="Output"/>
-    <tableColumn id="5" name="current post joining" dataDxfId="3" dataCellStyle="Output"/>
-    <tableColumn id="6" name="Study" dataDxfId="2" dataCellStyle="Output"/>
-    <tableColumn id="7" name="mobile no" dataDxfId="1"/>
+    <tableColumn id="1" name="SERIAL" dataDxfId="6" dataCellStyle="Output"/>
+    <tableColumn id="2" name="Name" dataDxfId="5" dataCellStyle="Output"/>
+    <tableColumn id="3" name="Post" dataDxfId="4"/>
+    <tableColumn id="4" name="Subject" dataDxfId="3" dataCellStyle="Output"/>
+    <tableColumn id="5" name="current post joining" dataDxfId="2" dataCellStyle="Output"/>
+    <tableColumn id="6" name="Study" dataDxfId="1" dataCellStyle="Output"/>
+    <tableColumn id="7" name="mobile no" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1054,893 +1060,1012 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="31.42578125" customWidth="1"/>
-    <col min="4" max="4" width="25.85546875" customWidth="1"/>
-    <col min="5" max="5" width="19.140625" customWidth="1"/>
-    <col min="6" max="6" width="20.85546875" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="4" width="31.42578125" customWidth="1"/>
+    <col min="5" max="5" width="25.85546875" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" customWidth="1"/>
+    <col min="7" max="7" width="20.85546875" customWidth="1"/>
+    <col min="8" max="8" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="C1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="E1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="F1" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="G1" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="H1" s="15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9">
+    <row r="2" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="9">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E2" s="4">
+      <c r="F2" s="4">
         <v>45044</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="G2" s="10">
+      <c r="H2" s="10">
         <v>9414894845</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9">
+    <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="9">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="5">
+      <c r="F3" s="5">
         <v>43262</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="10">
+      <c r="H3" s="10">
         <v>9950695755</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9">
+    <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="9">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>62</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>62</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="G4" s="10">
+      <c r="H4" s="10">
         <v>9460927989</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9">
+    <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="9">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="5">
+      <c r="F5" s="5">
         <v>42616</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="G5" s="10">
+      <c r="H5" s="10">
         <v>9024347777</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9">
+    <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="9">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E6" s="5">
+      <c r="F6" s="5">
         <v>46009</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G6" s="10">
+      <c r="H6" s="10">
         <v>9610817102</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9">
+    <row r="7" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="9">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="5">
+      <c r="F7" s="5">
         <v>42914</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G7" s="10">
+      <c r="H7" s="10">
         <v>8963892319</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9">
+    <row r="8" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="9">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="5">
+      <c r="F8" s="5">
         <v>42920</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="G8" s="10">
+      <c r="H8" s="10">
         <v>8118893102</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9">
+    <row r="9" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="9">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="4">
+      <c r="F9" s="4">
         <v>42581</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G9" s="10">
+      <c r="H9" s="10">
         <v>9057295392</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9">
+    <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="9">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="5">
+      <c r="F10" s="5">
         <v>45644</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G10" s="10">
+      <c r="H10" s="10">
         <v>9929189014</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9">
+    <row r="11" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="9">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="5">
+      <c r="F11" s="5">
         <v>45782</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G11" s="10">
+      <c r="H11" s="10">
         <v>9928267724</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9">
+    <row r="12" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="9">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E12" s="5">
+      <c r="F12" s="5">
         <v>42756</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G12" s="10">
+      <c r="H12" s="10">
         <v>9079682607</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="9">
+    <row r="13" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="9">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="D13" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="4">
+      <c r="F13" s="4">
         <v>44237</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="10">
+      <c r="H13" s="10">
         <v>9887653869</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="9">
+    <row r="14" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="9">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E14" s="4">
+      <c r="F14" s="4">
         <v>44275</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="G14" s="10">
+      <c r="H14" s="10">
         <v>9602203999</v>
       </c>
-      <c r="H14" s="1"/>
-    </row>
-    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="9">
+      <c r="I14" s="1"/>
+    </row>
+    <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="9">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="4">
+      <c r="F15" s="4">
         <v>43651</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G15" s="10">
+      <c r="H15" s="10">
         <v>9829990632</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9">
+    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="9">
+        <v>15</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="4">
+      <c r="F16" s="4">
         <v>42760</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G16" s="10">
+      <c r="H16" s="10">
         <v>9950361008</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9">
+    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="9">
+        <v>16</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="4">
+      <c r="F17" s="4">
         <v>43256</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G17" s="10">
+      <c r="H17" s="10">
         <v>9950541321</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="9">
+    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="9">
         <v>18</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E18" s="5">
+      <c r="F18" s="5">
         <v>45034</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G18" s="11">
+      <c r="H18" s="11">
         <v>9784730824</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9">
+    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="9">
         <v>19</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E19" s="5">
+      <c r="F19" s="5">
         <v>44981</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G19" s="10">
+      <c r="H19" s="10">
         <v>8562868641</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="9">
+    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="9">
         <v>20</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="4">
+      <c r="F20" s="4">
         <v>39465</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="G20" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G20" s="10">
+      <c r="H20" s="10">
         <v>9571894862</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9">
+    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="9">
         <v>21</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="4">
+      <c r="F21" s="4">
         <v>44468</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="G21" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G21" s="10">
+      <c r="H21" s="10">
         <v>7240106557</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="9">
+    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="9">
         <v>22</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="5">
+      <c r="F22" s="5">
         <v>44733</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="G22" s="10">
+      <c r="H22" s="10">
         <v>7877845982</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="9">
+    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="9">
         <v>23</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E23" s="4">
+      <c r="F23" s="4">
         <v>38439</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G23" s="10">
+      <c r="H23" s="10">
         <v>9982823574</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9">
+    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="9">
         <v>24</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="D24" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E24" s="4">
+      <c r="F24" s="4">
         <v>44828</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="G24" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G24" s="10">
+      <c r="H24" s="10">
         <v>8619212002</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="9">
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="9">
         <v>25</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="C25" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="E25" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E25" s="7">
+      <c r="F25" s="7">
         <v>41943</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="G25" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="G25" s="10">
+      <c r="H25" s="10">
         <v>9887128681</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="9">
+    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="9">
         <v>26</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="D26" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="E26" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="4">
+      <c r="F26" s="4">
         <v>34232</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="G26" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="G26" s="10">
+      <c r="H26" s="10">
         <v>7568392031</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="9">
+    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="9">
         <v>27</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="D27" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="E27" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E27" s="5">
+      <c r="F27" s="5">
         <v>35097</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="G27" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G27" s="12">
+      <c r="H27" s="12">
         <v>9887340355</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="9">
+    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="9">
         <v>28</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="D28" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="E28" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E28" s="5">
+      <c r="F28" s="5">
         <v>38901</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="G28" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="G28" s="10">
+      <c r="H28" s="10">
         <v>9982845457</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9">
+    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="9">
         <v>29</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="D29" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="E29" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E29" s="4">
+      <c r="F29" s="4">
         <v>35614</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="G29" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="G29" s="10">
+      <c r="H29" s="10">
         <v>7737062475</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9">
+    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" s="9">
         <v>30</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="C30" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="D30" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="E30" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E30" s="5">
+      <c r="F30" s="5">
         <v>34059</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="G30" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="G30" s="10">
+      <c r="H30" s="10">
         <v>9460505720</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9">
+    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" s="9">
         <v>31</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="D31" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E31" s="5">
+      <c r="F31" s="5">
         <v>38561</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="G31" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="G31" s="10">
+      <c r="H31" s="10">
         <v>9145836326</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="9">
+    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" s="9">
         <v>32</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="D32" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="E32" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E32" s="5">
+      <c r="F32" s="5">
         <v>39662</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="G32" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G32" s="10">
+      <c r="H32" s="10">
         <v>9784431932</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="9">
+    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" s="9">
         <v>33</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="D33" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="E33" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="E33" s="5">
+      <c r="F33" s="5">
         <v>39198</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="G33" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="G33" s="10">
+      <c r="H33" s="10">
         <v>9887124545</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="9">
+    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" s="9">
         <v>34</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="D34" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="E34" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E34" s="8">
+      <c r="F34" s="8">
         <v>42086</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="G34" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="G34" s="10">
+      <c r="H34" s="10">
         <v>8094023875</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="9">
+    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" s="9">
         <v>35</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="D35" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E35" s="5">
+      <c r="F35" s="5">
         <v>42086</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="G35" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G35" s="10">
+      <c r="H35" s="10">
         <v>9950731013</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="9">
+    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" s="9">
         <v>36</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="D36" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E36" s="5">
+      <c r="F36" s="5">
         <v>38447</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="G36" s="10">
+      <c r="H36" s="10">
         <v>9928511626</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="9">
+    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" s="9">
         <v>37</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="D37" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="E37" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E37" s="5">
+      <c r="F37" s="5">
         <v>45069</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="G37" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="G37" s="10">
+      <c r="H37" s="10">
         <v>8290730037</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="16">
+    <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" s="16">
         <v>38</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="C38" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="C38" s="18" t="s">
+      <c r="D38" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="E38" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="E38" s="19">
+      <c r="F38" s="20">
         <v>44733</v>
       </c>
-      <c r="F38" s="17" t="s">
+      <c r="G38" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="G38" s="20">
+      <c r="H38" s="19">
         <v>9887607170</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:A38">
+    <sortState ref="A2:A38">
+      <sortCondition ref="A1:A38"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix: Update mobile number for #34 Dipankar Sharma to 9309348008
</commit_message>
<xml_diff>
--- a/staff/staff details.xlsx
+++ b/staff/staff details.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="91">
   <si>
     <t>SERIAL</t>
   </si>
@@ -289,6 +289,9 @@
   </si>
   <si>
     <t>DEVKI NANDAN SHARMA</t>
+  </si>
+  <si>
+    <t>Political Science(Art)</t>
   </si>
 </sst>
 </file>
@@ -719,6 +722,15 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -726,15 +738,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -773,7 +776,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:G38" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7" headerRowCellStyle="Output">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:G38" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8" totalsRowBorderDxfId="7" headerRowCellStyle="Output">
   <autoFilter ref="A1:G38"/>
   <sortState ref="A2:G38">
     <sortCondition ref="A1:A38"/>
@@ -1261,13 +1264,13 @@
         <v>16</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="E9" s="10">
         <v>43262</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="G9" s="8">
         <v>9950695755</v>
@@ -1869,7 +1872,7 @@
         <v>62</v>
       </c>
       <c r="G35" s="8">
-        <v>8619212002</v>
+        <v>9309348008</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: configure student import and export format to 11 fields (Class, Section, SRNO, Rollno, Student Name, Father/Guardian Name, Mother Name, Cast Category, Gender, DOB, Mobile No)
</commit_message>
<xml_diff>
--- a/staff/staff details.xlsx
+++ b/staff/staff details.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="91">
   <si>
     <t>SERIAL</t>
   </si>
@@ -90,9 +90,6 @@
     <t>RAMESH KUMAR</t>
   </si>
   <si>
-    <t>Physics (Science Stream)</t>
-  </si>
-  <si>
     <t>B.SC/M.SC/B.ED</t>
   </si>
   <si>
@@ -114,9 +111,6 @@
     <t>KANHAIYA LAL SHARMA</t>
   </si>
   <si>
-    <t>Chemistry (Science Stream)</t>
-  </si>
-  <si>
     <t>B.SC/M.SC/B.ED/RSCIT</t>
   </si>
   <si>
@@ -132,9 +126,6 @@
     <t>MANOJ KUMAR SARSWAT</t>
   </si>
   <si>
-    <t>Biology (Science Stream)</t>
-  </si>
-  <si>
     <t>TILOKA RAM DUDI</t>
   </si>
   <si>
@@ -168,9 +159,6 @@
     <t>Senior Computer Instructor</t>
   </si>
   <si>
-    <t>COMPUTER (Science Stream)</t>
-  </si>
-  <si>
     <t>BCA/MCA</t>
   </si>
   <si>
@@ -204,9 +192,6 @@
     <t>DHARMPAL BUGALIA</t>
   </si>
   <si>
-    <t>Mathematics/ Science</t>
-  </si>
-  <si>
     <t>B.SC/B.ED</t>
   </si>
   <si>
@@ -291,7 +276,22 @@
     <t>DEVKI NANDAN SHARMA</t>
   </si>
   <si>
-    <t>Political Science(Art)</t>
+    <t xml:space="preserve">Chemistry </t>
+  </si>
+  <si>
+    <t>Biology</t>
+  </si>
+  <si>
+    <t>COMPUTER</t>
+  </si>
+  <si>
+    <t>Physics</t>
+  </si>
+  <si>
+    <t>Faculty</t>
+  </si>
+  <si>
+    <t>Joining</t>
   </si>
 </sst>
 </file>
@@ -557,7 +557,43 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="13">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -776,19 +812,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:G38" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8" totalsRowBorderDxfId="7" headerRowCellStyle="Output">
-  <autoFilter ref="A1:G38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I38" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9" headerRowCellStyle="Output">
+  <autoFilter ref="A1:I38"/>
   <sortState ref="A2:G38">
     <sortCondition ref="A1:A38"/>
   </sortState>
-  <tableColumns count="7">
-    <tableColumn id="1" name="SERIAL" dataDxfId="6" dataCellStyle="Output"/>
-    <tableColumn id="2" name="Name" dataDxfId="5" dataCellStyle="Output"/>
-    <tableColumn id="3" name="Post" dataDxfId="4"/>
-    <tableColumn id="4" name="Subject" dataDxfId="3" dataCellStyle="Output"/>
-    <tableColumn id="5" name="current post joining" dataDxfId="2" dataCellStyle="Output"/>
-    <tableColumn id="6" name="Study" dataDxfId="1" dataCellStyle="Output"/>
-    <tableColumn id="7" name="mobile no" dataDxfId="0"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="SERIAL" dataDxfId="8" dataCellStyle="Output"/>
+    <tableColumn id="2" name="Name" dataDxfId="7" dataCellStyle="Output"/>
+    <tableColumn id="3" name="Post" dataDxfId="6"/>
+    <tableColumn id="4" name="Subject" dataDxfId="5" dataCellStyle="Output"/>
+    <tableColumn id="8" name="Faculty" dataDxfId="1" dataCellStyle="Output"/>
+    <tableColumn id="9" name="Joining" dataDxfId="0" dataCellStyle="Output"/>
+    <tableColumn id="5" name="current post joining" dataDxfId="4" dataCellStyle="Output"/>
+    <tableColumn id="6" name="Study" dataDxfId="3" dataCellStyle="Output"/>
+    <tableColumn id="7" name="mobile no" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1057,19 +1095,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
     <col min="2" max="2" width="25.140625" customWidth="1"/>
     <col min="3" max="3" width="22.7109375" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" customWidth="1"/>
-    <col min="6" max="6" width="20.85546875" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="4" max="6" width="22.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.85546875" customWidth="1"/>
+    <col min="9" max="9" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1083,16 +1121,22 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1105,17 +1149,19 @@
       <c r="D2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="7">
         <v>45044</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="8">
+      <c r="I2" s="8">
         <v>9414894845</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1128,17 +1174,19 @@
       <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="7">
         <v>42581</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="8">
+      <c r="I3" s="8">
         <v>9057295392</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1151,17 +1199,19 @@
       <c r="D4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="10">
-        <v>46294</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="10">
+        <v>45929</v>
+      </c>
+      <c r="H4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="8">
+      <c r="I4" s="8">
         <v>9460927989</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1174,17 +1224,19 @@
       <c r="D5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="10">
         <v>42616</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="8">
+      <c r="I5" s="8">
         <v>9024347777</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1197,17 +1249,19 @@
       <c r="D6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="10">
         <v>42756</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="8">
+      <c r="I6" s="8">
         <v>9079682607</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1218,116 +1272,126 @@
         <v>16</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="10">
+        <v>42914</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="10">
-        <v>42914</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="8">
+      <c r="I7" s="8">
         <v>8963892319</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="10">
+        <v>42920</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="10">
-        <v>42920</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="8">
+      <c r="I8" s="8">
         <v>8118893102</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="E9" s="10">
+        <v>20</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="10">
         <v>43262</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="H9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="8">
+      <c r="I9" s="8">
         <v>9950695755</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="7">
+        <v>85</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="7">
         <v>44237</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G10" s="8">
+      <c r="H10" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="8">
         <v>9887653869</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="7">
+        <v>32</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="7">
         <v>44275</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="8">
+      <c r="H11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" s="8">
         <v>9602203999</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>16</v>
@@ -1335,612 +1399,666 @@
       <c r="D12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="10">
         <v>45644</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="8">
+      <c r="I12" s="8">
         <v>9929189014</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="10">
+        <v>86</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="10">
         <v>45782</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G13" s="8">
+      <c r="H13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="8">
         <v>9928267724</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>16</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="10">
+        <v>25</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="10">
         <v>46009</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G14" s="8">
+      <c r="I14" s="8">
         <v>9610817102</v>
       </c>
-      <c r="H14" s="11"/>
-    </row>
-    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J14" s="11"/>
+    </row>
+    <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E15" s="7">
+        <v>38</v>
+      </c>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="7">
         <v>42760</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G15" s="8">
+      <c r="H15" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I15" s="8">
         <v>9950361008</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="E16" s="7">
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="7">
         <v>43256</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G16" s="8">
+      <c r="H16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I16" s="8">
         <v>9950541321</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>16</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" s="7">
+        <v>42</v>
+      </c>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="7">
         <v>43651</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="G17" s="8">
+      <c r="H17" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I17" s="8">
         <v>9829990632</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>17</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E18" s="10">
+        <v>87</v>
+      </c>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="10">
         <v>44981</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="G18" s="8">
+      <c r="H18" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I18" s="8">
         <v>8562868641</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>18</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="10">
         <v>34059</v>
       </c>
-      <c r="F19" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G19" s="8">
+      <c r="H19" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I19" s="8">
         <v>9460505720</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="7">
         <v>34232</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G20" s="8">
+      <c r="H20" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I20" s="8">
         <v>7568392031</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>20</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E21" s="10">
+        <v>53</v>
+      </c>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="10">
         <v>35097</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="H21" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G21" s="12">
+      <c r="I21" s="12">
         <v>9887340355</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>21</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E22" s="7">
+        <v>53</v>
+      </c>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="7">
         <v>35614</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="G22" s="8">
+      <c r="H22" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="I22" s="8">
         <v>7737062475</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>22</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E23" s="7">
+        <v>42</v>
+      </c>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="7">
         <v>38439</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="G23" s="8">
+      <c r="H23" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I23" s="8">
         <v>9982823574</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>23</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="E24" s="10">
+        <v>40</v>
+      </c>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="10">
         <v>38447</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G24" s="8">
+      <c r="H24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I24" s="8">
         <v>9928511626</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>24</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E25" s="10">
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="10">
         <v>38901</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="G25" s="8">
+      <c r="H25" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="I25" s="8">
         <v>9982845457</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>25</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="E26" s="10">
+        <v>62</v>
+      </c>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="10">
         <v>39198</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G26" s="8">
+      <c r="H26" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I26" s="8">
         <v>9887124545</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>26</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="E27" s="7">
+        <v>62</v>
+      </c>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="7">
         <v>39465</v>
       </c>
-      <c r="F27" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G27" s="8">
+      <c r="H27" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I27" s="8">
         <v>9571894862</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>27</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" s="10">
+        <v>42</v>
+      </c>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="10">
         <v>39662</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="G28" s="8">
+      <c r="H28" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I28" s="8">
         <v>9784431932</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>28</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E29" s="13">
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="13">
         <v>42086</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="G29" s="8">
+      <c r="H29" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="I29" s="8">
         <v>8094023875</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>29</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E30" s="10">
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="10">
         <v>42086</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="G30" s="8">
+      <c r="H30" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="I30" s="8">
         <v>9950731013</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>30</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E31" s="10">
+        <v>87</v>
+      </c>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="10">
         <v>45034</v>
       </c>
-      <c r="F31" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="G31" s="14">
+      <c r="H31" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I31" s="14">
         <v>9784730824</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>31</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E32" s="15">
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="15">
         <v>41943</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="H32" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G32" s="8">
+      <c r="I32" s="8">
         <v>9887128681</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>32</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E33" s="7">
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="7">
         <v>44468</v>
       </c>
-      <c r="F33" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="G33" s="8">
+      <c r="H33" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="I33" s="8">
         <v>7240106557</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>33</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E34" s="10">
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="10">
         <v>44733</v>
       </c>
-      <c r="F34" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="G34" s="8">
+      <c r="H34" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="I34" s="8">
         <v>7877845982</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <v>34</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E35" s="7">
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="7">
         <v>44828</v>
       </c>
-      <c r="F35" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="G35" s="8">
+      <c r="H35" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I35" s="8">
         <v>9309348008</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>35</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E36" s="10">
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="10">
         <v>45069</v>
       </c>
-      <c r="F36" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="G36" s="8">
+      <c r="H36" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="I36" s="8">
         <v>8290730037</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>36</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E37" s="10">
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="10">
         <v>38561</v>
       </c>
-      <c r="F37" s="6" t="s">
+      <c r="H37" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G37" s="8">
+      <c r="I37" s="8">
         <v>9145836326</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="16">
         <v>37</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D38" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="E38" s="19">
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="19">
         <v>46194</v>
       </c>
-      <c r="F38" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="G38" s="20">
+      <c r="H38" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="I38" s="20">
         <v>9887607170</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: student confidentiality protection, 11-column student format, and excel (.xlsx) import/export for students, teachers, and results
</commit_message>
<xml_diff>
--- a/staff/staff details.xlsx
+++ b/staff/staff details.xlsx
@@ -298,7 +298,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -333,6 +333,14 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -512,7 +520,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -552,48 +560,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
   <dxfs count="13">
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -645,6 +620,42 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -822,11 +833,11 @@
     <tableColumn id="2" name="Name" dataDxfId="7" dataCellStyle="Output"/>
     <tableColumn id="3" name="Post" dataDxfId="6"/>
     <tableColumn id="4" name="Subject" dataDxfId="5" dataCellStyle="Output"/>
-    <tableColumn id="8" name="Faculty" dataDxfId="1" dataCellStyle="Output"/>
-    <tableColumn id="9" name="Joining" dataDxfId="0" dataCellStyle="Output"/>
-    <tableColumn id="5" name="current post joining" dataDxfId="4" dataCellStyle="Output"/>
-    <tableColumn id="6" name="Study" dataDxfId="3" dataCellStyle="Output"/>
-    <tableColumn id="7" name="mobile no" dataDxfId="2"/>
+    <tableColumn id="8" name="Faculty" dataDxfId="4" dataCellStyle="Output"/>
+    <tableColumn id="9" name="Joining" dataDxfId="3" dataCellStyle="Output"/>
+    <tableColumn id="5" name="current post joining" dataDxfId="2" dataCellStyle="Output"/>
+    <tableColumn id="6" name="Study" dataDxfId="1" dataCellStyle="Output"/>
+    <tableColumn id="7" name="mobile no" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1176,8 +1187,8 @@
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="7">
-        <v>42581</v>
+      <c r="G3" s="10">
+        <v>45929</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>12</v>
@@ -1215,7 +1226,7 @@
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="21" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -1265,7 +1276,7 @@
       <c r="A7" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="21" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -1716,7 +1727,7 @@
       <c r="A25" s="4">
         <v>24</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="21" t="s">
         <v>59</v>
       </c>
       <c r="C25" s="9" t="s">
@@ -2064,8 +2075,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update staff details with accurate experience and restrict faculties strictly to Arts, Science, and Administration
</commit_message>
<xml_diff>
--- a/staff/staff details.xlsx
+++ b/staff/staff details.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="90">
   <si>
     <t>SERIAL</t>
   </si>
@@ -172,9 +172,6 @@
   </si>
   <si>
     <t>KANCHAN LATA PUROHIT</t>
-  </si>
-  <si>
-    <t>KANHAIYA LAL JANGID</t>
   </si>
   <si>
     <t>Teacher Level-2</t>
@@ -1132,10 +1129,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>4</v>
@@ -1283,7 +1280,7 @@
         <v>16</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
@@ -1358,7 +1355,7 @@
         <v>16</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
@@ -1433,7 +1430,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
@@ -1559,7 +1556,7 @@
         <v>45</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
@@ -1624,42 +1621,28 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4">
-        <v>20</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="A21" s="4"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
-      <c r="G21" s="10">
-        <v>35097</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="I21" s="12">
-        <v>9887340355</v>
-      </c>
+      <c r="G21" s="10"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="12"/>
     </row>
     <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>21</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C22" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>53</v>
       </c>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
@@ -1667,7 +1650,7 @@
         <v>35614</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I22" s="8">
         <v>7737062475</v>
@@ -1678,10 +1661,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>42</v>
@@ -1692,7 +1675,7 @@
         <v>38439</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I23" s="8">
         <v>9982823574</v>
@@ -1703,10 +1686,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>40</v>
@@ -1728,7 +1711,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>48</v>
@@ -1742,7 +1725,7 @@
         <v>38901</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I25" s="8">
         <v>9982845457</v>
@@ -1753,13 +1736,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>62</v>
       </c>
       <c r="E26" s="6"/>
       <c r="F26" s="6"/>
@@ -1778,13 +1761,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="6"/>
@@ -1803,10 +1786,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>42</v>
@@ -1817,7 +1800,7 @@
         <v>39662</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I28" s="8">
         <v>9784431932</v>
@@ -1828,7 +1811,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>48</v>
@@ -1842,7 +1825,7 @@
         <v>42086</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I29" s="8">
         <v>8094023875</v>
@@ -1853,7 +1836,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>48</v>
@@ -1867,7 +1850,7 @@
         <v>42086</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I30" s="8">
         <v>9950731013</v>
@@ -1878,13 +1861,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>70</v>
-      </c>
       <c r="D31" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E31" s="5"/>
       <c r="F31" s="5"/>
@@ -1903,10 +1886,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="9" t="s">
         <v>71</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>72</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>9</v>
@@ -1928,10 +1911,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C33" s="9" t="s">
         <v>73</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>74</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>9</v>
@@ -1942,7 +1925,7 @@
         <v>44468</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I33" s="8">
         <v>7240106557</v>
@@ -1953,10 +1936,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="9" t="s">
         <v>76</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>77</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>9</v>
@@ -1967,7 +1950,7 @@
         <v>44733</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I34" s="8">
         <v>7877845982</v>
@@ -1978,10 +1961,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>9</v>
@@ -1992,7 +1975,7 @@
         <v>44828</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I35" s="8">
         <v>9309348008</v>
@@ -2003,10 +1986,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>9</v>
@@ -2017,7 +2000,7 @@
         <v>45069</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I36" s="8">
         <v>8290730037</v>
@@ -2028,10 +2011,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C37" s="9" t="s">
         <v>82</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>83</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>9</v>
@@ -2053,10 +2036,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D38" s="17" t="s">
         <v>9</v>
@@ -2067,7 +2050,7 @@
         <v>46194</v>
       </c>
       <c r="H38" s="17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I38" s="20">
         <v>9887607170</v>

</xml_diff>